<commit_message>
cleaned wind noise model, added price setter print
</commit_message>
<xml_diff>
--- a/simple_market_clearing/clearing_analysis.xlsx
+++ b/simple_market_clearing/clearing_analysis.xlsx
@@ -597,10 +597,10 @@
         <v>50.0</v>
       </c>
       <c r="E9">
-        <v>214.67</v>
+        <v>194.71</v>
       </c>
       <c r="F9">
-        <v>214.67</v>
+        <v>194.71</v>
       </c>
       <c r="G9">
         <v>0.0</v>
@@ -666,10 +666,10 @@
         <v>50.0</v>
       </c>
       <c r="E12">
-        <v>170.01</v>
+        <v>226.04</v>
       </c>
       <c r="F12">
-        <v>170.01</v>
+        <v>226.04</v>
       </c>
       <c r="G12">
         <v>0.0</v>
@@ -735,10 +735,10 @@
         <v>50.0</v>
       </c>
       <c r="E15">
-        <v>317.56</v>
+        <v>220.88</v>
       </c>
       <c r="F15">
-        <v>317.56</v>
+        <v>220.88</v>
       </c>
       <c r="G15">
         <v>0.0</v>
@@ -804,10 +804,10 @@
         <v>50.0</v>
       </c>
       <c r="E18">
-        <v>240.68</v>
+        <v>303.74</v>
       </c>
       <c r="F18">
-        <v>240.68</v>
+        <v>303.74</v>
       </c>
       <c r="G18">
         <v>0.0</v>
@@ -873,10 +873,10 @@
         <v>50.0</v>
       </c>
       <c r="E21">
-        <v>367.61</v>
+        <v>366.04</v>
       </c>
       <c r="F21">
-        <v>367.61</v>
+        <v>366.04</v>
       </c>
       <c r="G21">
         <v>0.0</v>
@@ -942,10 +942,10 @@
         <v>50.0</v>
       </c>
       <c r="E24">
-        <v>402.05</v>
+        <v>403.06</v>
       </c>
       <c r="F24">
-        <v>402.05</v>
+        <v>403.06</v>
       </c>
       <c r="G24">
         <v>0.0</v>
@@ -988,10 +988,10 @@
         <v>100.0</v>
       </c>
       <c r="E26">
-        <v>-0.0</v>
+        <v>291.21</v>
       </c>
       <c r="F26">
-        <v>0.0</v>
+        <v>291.21</v>
       </c>
       <c r="G26">
         <v>0.0</v>
@@ -1011,10 +1011,10 @@
         <v>100.0</v>
       </c>
       <c r="E27">
-        <v>560.98</v>
+        <v>508.79</v>
       </c>
       <c r="F27">
-        <v>560.98</v>
+        <v>508.79</v>
       </c>
       <c r="G27">
         <v>0.0</v>
@@ -1057,10 +1057,10 @@
         <v>100.0</v>
       </c>
       <c r="E29">
-        <v>406.13</v>
+        <v>354.22</v>
       </c>
       <c r="F29">
-        <v>406.13</v>
+        <v>354.22</v>
       </c>
       <c r="G29">
         <v>0.0</v>
@@ -1080,10 +1080,10 @@
         <v>100.0</v>
       </c>
       <c r="E30">
-        <v>593.87</v>
+        <v>645.78</v>
       </c>
       <c r="F30">
-        <v>593.87</v>
+        <v>645.78</v>
       </c>
       <c r="G30">
         <v>0.0</v>
@@ -1126,10 +1126,10 @@
         <v>100.0</v>
       </c>
       <c r="E32">
-        <v>324.99</v>
+        <v>289.03</v>
       </c>
       <c r="F32">
-        <v>324.99</v>
+        <v>289.03</v>
       </c>
       <c r="G32">
         <v>0.0</v>
@@ -1149,10 +1149,10 @@
         <v>100.0</v>
       </c>
       <c r="E33">
-        <v>375.01</v>
+        <v>410.97</v>
       </c>
       <c r="F33">
-        <v>375.01</v>
+        <v>410.97</v>
       </c>
       <c r="G33">
         <v>0.0</v>
@@ -1195,10 +1195,10 @@
         <v>100.0</v>
       </c>
       <c r="E35">
-        <v>198.23</v>
+        <v>60.69</v>
       </c>
       <c r="F35">
-        <v>198.23</v>
+        <v>60.69</v>
       </c>
       <c r="G35">
         <v>0.0</v>
@@ -1218,10 +1218,10 @@
         <v>100.0</v>
       </c>
       <c r="E36">
-        <v>329.77</v>
+        <v>319.31</v>
       </c>
       <c r="F36">
-        <v>329.77</v>
+        <v>319.31</v>
       </c>
       <c r="G36">
         <v>0.0</v>
@@ -1264,10 +1264,10 @@
         <v>100.0</v>
       </c>
       <c r="E38">
-        <v>573.61</v>
+        <v>57.25</v>
       </c>
       <c r="F38">
-        <v>573.61</v>
+        <v>57.25</v>
       </c>
       <c r="G38">
         <v>0.0</v>
@@ -1287,10 +1287,10 @@
         <v>100.0</v>
       </c>
       <c r="E39">
-        <v>226.39</v>
+        <v>342.75</v>
       </c>
       <c r="F39">
-        <v>226.39</v>
+        <v>342.75</v>
       </c>
       <c r="G39">
         <v>0.0</v>
@@ -1333,10 +1333,10 @@
         <v>100.0</v>
       </c>
       <c r="E41">
-        <v>369.86</v>
+        <v>442.47</v>
       </c>
       <c r="F41">
-        <v>369.86</v>
+        <v>442.47</v>
       </c>
       <c r="G41">
         <v>0.0</v>
@@ -1356,10 +1356,10 @@
         <v>100.0</v>
       </c>
       <c r="E42">
-        <v>330.14</v>
+        <v>257.53</v>
       </c>
       <c r="F42">
-        <v>330.14</v>
+        <v>257.53</v>
       </c>
       <c r="G42">
         <v>0.0</v>
@@ -1402,10 +1402,10 @@
         <v>100.0</v>
       </c>
       <c r="E44">
-        <v>238.44</v>
+        <v>311.17</v>
       </c>
       <c r="F44">
-        <v>238.44</v>
+        <v>311.17</v>
       </c>
       <c r="G44">
         <v>0.0</v>
@@ -1425,10 +1425,10 @@
         <v>100.0</v>
       </c>
       <c r="E45">
-        <v>361.56</v>
+        <v>288.83</v>
       </c>
       <c r="F45">
-        <v>361.56</v>
+        <v>288.83</v>
       </c>
       <c r="G45">
         <v>0.0</v>
@@ -1471,10 +1471,10 @@
         <v>100.0</v>
       </c>
       <c r="E47">
-        <v>458.97</v>
+        <v>427.04</v>
       </c>
       <c r="F47">
-        <v>458.97</v>
+        <v>427.04</v>
       </c>
       <c r="G47">
         <v>0.0</v>
@@ -1494,10 +1494,10 @@
         <v>100.0</v>
       </c>
       <c r="E48">
-        <v>241.03</v>
+        <v>272.96</v>
       </c>
       <c r="F48">
-        <v>241.03</v>
+        <v>272.96</v>
       </c>
       <c r="G48">
         <v>0.0</v>
@@ -1540,10 +1540,10 @@
         <v>100.0</v>
       </c>
       <c r="E50">
-        <v>534.68</v>
+        <v>535.41</v>
       </c>
       <c r="F50">
-        <v>534.68</v>
+        <v>535.41</v>
       </c>
       <c r="G50">
         <v>0.0</v>
@@ -1563,10 +1563,10 @@
         <v>100.0</v>
       </c>
       <c r="E51">
-        <v>165.32</v>
+        <v>164.59</v>
       </c>
       <c r="F51">
-        <v>165.32</v>
+        <v>164.59</v>
       </c>
       <c r="G51">
         <v>0.0</v>
@@ -1609,10 +1609,10 @@
         <v>100.0</v>
       </c>
       <c r="E53">
-        <v>463.16</v>
+        <v>522.53</v>
       </c>
       <c r="F53">
-        <v>463.16</v>
+        <v>522.53</v>
       </c>
       <c r="G53">
         <v>0.0</v>
@@ -1632,10 +1632,10 @@
         <v>100.0</v>
       </c>
       <c r="E54">
-        <v>236.84</v>
+        <v>177.47</v>
       </c>
       <c r="F54">
-        <v>236.84</v>
+        <v>177.47</v>
       </c>
       <c r="G54">
         <v>0.0</v>
@@ -1678,10 +1678,10 @@
         <v>100.0</v>
       </c>
       <c r="E56">
-        <v>181.76</v>
+        <v>177.48</v>
       </c>
       <c r="F56">
-        <v>181.76</v>
+        <v>177.48</v>
       </c>
       <c r="G56">
         <v>0.0</v>
@@ -1701,10 +1701,10 @@
         <v>100.0</v>
       </c>
       <c r="E57">
-        <v>718.24</v>
+        <v>722.52</v>
       </c>
       <c r="F57">
-        <v>718.24</v>
+        <v>722.52</v>
       </c>
       <c r="G57">
         <v>0.0</v>
@@ -1747,10 +1747,10 @@
         <v>100.0</v>
       </c>
       <c r="E59">
-        <v>-0.0</v>
+        <v>182.1</v>
       </c>
       <c r="F59">
-        <v>0.0</v>
+        <v>182.1</v>
       </c>
       <c r="G59">
         <v>0.0</v>
@@ -1770,10 +1770,10 @@
         <v>100.0</v>
       </c>
       <c r="E60">
-        <v>691.03</v>
+        <v>817.9</v>
       </c>
       <c r="F60">
-        <v>691.03</v>
+        <v>817.9</v>
       </c>
       <c r="G60">
         <v>0.0</v>
@@ -1816,10 +1816,10 @@
         <v>100.0</v>
       </c>
       <c r="E62">
-        <v>193.58</v>
+        <v>245.57</v>
       </c>
       <c r="F62">
-        <v>193.58</v>
+        <v>245.57</v>
       </c>
       <c r="G62">
         <v>0.0</v>
@@ -1839,10 +1839,10 @@
         <v>100.0</v>
       </c>
       <c r="E63">
-        <v>906.42</v>
+        <v>854.43</v>
       </c>
       <c r="F63">
-        <v>906.42</v>
+        <v>854.43</v>
       </c>
       <c r="G63">
         <v>0.0</v>
@@ -1885,10 +1885,10 @@
         <v>100.0</v>
       </c>
       <c r="E65">
-        <v>169.5</v>
+        <v>176.27</v>
       </c>
       <c r="F65">
-        <v>169.5</v>
+        <v>176.27</v>
       </c>
       <c r="G65">
         <v>0.0</v>
@@ -1908,10 +1908,10 @@
         <v>100.0</v>
       </c>
       <c r="E66">
-        <v>830.5</v>
+        <v>823.73</v>
       </c>
       <c r="F66">
-        <v>830.5</v>
+        <v>823.73</v>
       </c>
       <c r="G66">
         <v>0.0</v>
@@ -1977,10 +1977,10 @@
         <v>50.0</v>
       </c>
       <c r="E69">
-        <v>825.6</v>
+        <v>723.44</v>
       </c>
       <c r="F69">
-        <v>825.6</v>
+        <v>723.44</v>
       </c>
       <c r="G69">
         <v>0.0</v>
@@ -2046,10 +2046,10 @@
         <v>50.0</v>
       </c>
       <c r="E72">
-        <v>676.87</v>
+        <v>689.92</v>
       </c>
       <c r="F72">
-        <v>676.87</v>
+        <v>689.92</v>
       </c>
       <c r="G72">
         <v>0.0</v>
@@ -2115,10 +2115,10 @@
         <v>50.0</v>
       </c>
       <c r="E75">
-        <v>562.08</v>
+        <v>603.0</v>
       </c>
       <c r="F75">
-        <v>562.08</v>
+        <v>603.0</v>
       </c>
       <c r="G75">
         <v>0.0</v>
@@ -2193,7 +2193,7 @@
         <v>5</v>
       </c>
       <c r="C5">
-        <v>83.39</v>
+        <v>125.0</v>
       </c>
       <c r="D5">
         <v>100.0</v>
@@ -2202,7 +2202,7 @@
         <v>-0.0</v>
       </c>
       <c r="F5">
-        <v>83.39</v>
+        <v>125.0</v>
       </c>
       <c r="G5">
         <v>-0.0</v>
@@ -2216,7 +2216,7 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>339.47</v>
+        <v>284.34</v>
       </c>
       <c r="D6">
         <v>100.0</v>
@@ -2225,7 +2225,7 @@
         <v>-0.0</v>
       </c>
       <c r="F6">
-        <v>339.47</v>
+        <v>284.34</v>
       </c>
       <c r="G6">
         <v>-0.0</v>
@@ -2262,19 +2262,19 @@
         <v>5</v>
       </c>
       <c r="C8">
-        <v>421.71</v>
+        <v>299.98</v>
       </c>
       <c r="D8">
         <v>100.0</v>
       </c>
       <c r="E8">
-        <v>-239.91</v>
+        <v>-96.3</v>
       </c>
       <c r="F8">
-        <v>181.8</v>
+        <v>203.68</v>
       </c>
       <c r="G8">
-        <v>-56.9</v>
+        <v>-32.1</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2285,19 +2285,19 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <v>178.29</v>
+        <v>300.02</v>
       </c>
       <c r="D9">
         <v>100.0</v>
       </c>
       <c r="E9">
-        <v>51.36</v>
+        <v>-44.59</v>
       </c>
       <c r="F9">
-        <v>229.65</v>
+        <v>255.43</v>
       </c>
       <c r="G9">
-        <v>28.8</v>
+        <v>-14.9</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2331,19 +2331,19 @@
         <v>5</v>
       </c>
       <c r="C11">
-        <v>475.66</v>
+        <v>499.69</v>
       </c>
       <c r="D11">
         <v>100.0</v>
       </c>
       <c r="E11">
-        <v>-17.98</v>
+        <v>-50.29</v>
       </c>
       <c r="F11">
-        <v>457.68</v>
+        <v>449.4</v>
       </c>
       <c r="G11">
-        <v>-3.8</v>
+        <v>-10.1</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2354,19 +2354,19 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>224.34</v>
+        <v>200.31</v>
       </c>
       <c r="D12">
         <v>100.0</v>
       </c>
       <c r="E12">
-        <v>17.98</v>
+        <v>50.29</v>
       </c>
       <c r="F12">
-        <v>242.32</v>
+        <v>250.6</v>
       </c>
       <c r="G12">
-        <v>8.0</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2400,19 +2400,19 @@
         <v>5</v>
       </c>
       <c r="C14">
-        <v>557.42</v>
+        <v>502.86</v>
       </c>
       <c r="D14">
         <v>100.0</v>
       </c>
       <c r="E14">
-        <v>66.93</v>
+        <v>36.04</v>
       </c>
       <c r="F14">
-        <v>624.36</v>
+        <v>538.91</v>
       </c>
       <c r="G14">
-        <v>12.0</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2423,19 +2423,19 @@
         <v>6</v>
       </c>
       <c r="C15">
-        <v>142.58</v>
+        <v>197.14</v>
       </c>
       <c r="D15">
         <v>100.0</v>
       </c>
       <c r="E15">
-        <v>-66.93</v>
+        <v>-36.04</v>
       </c>
       <c r="F15">
-        <v>75.64</v>
+        <v>161.09</v>
       </c>
       <c r="G15">
-        <v>-46.9</v>
+        <v>-18.3</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2469,19 +2469,19 @@
         <v>5</v>
       </c>
       <c r="C17">
-        <v>454.01</v>
+        <v>506.5</v>
       </c>
       <c r="D17">
         <v>100.0</v>
       </c>
       <c r="E17">
-        <v>20.1</v>
+        <v>-92.88</v>
       </c>
       <c r="F17">
-        <v>474.11</v>
+        <v>413.62</v>
       </c>
       <c r="G17">
-        <v>4.4</v>
+        <v>-18.3</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2492,19 +2492,19 @@
         <v>6</v>
       </c>
       <c r="C18">
-        <v>245.99</v>
+        <v>193.5</v>
       </c>
       <c r="D18">
         <v>100.0</v>
       </c>
       <c r="E18">
-        <v>-20.1</v>
+        <v>92.88</v>
       </c>
       <c r="F18">
-        <v>225.89</v>
+        <v>286.38</v>
       </c>
       <c r="G18">
-        <v>-8.2</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -2538,19 +2538,19 @@
         <v>5</v>
       </c>
       <c r="C20">
-        <v>135.25</v>
+        <v>212.57</v>
       </c>
       <c r="D20">
         <v>100.0</v>
       </c>
       <c r="E20">
-        <v>16.09</v>
+        <v>-31.51</v>
       </c>
       <c r="F20">
-        <v>151.34</v>
+        <v>181.06</v>
       </c>
       <c r="G20">
-        <v>11.9</v>
+        <v>-14.8</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2561,19 +2561,19 @@
         <v>6</v>
       </c>
       <c r="C21">
-        <v>764.75</v>
+        <v>687.43</v>
       </c>
       <c r="D21">
         <v>100.0</v>
       </c>
       <c r="E21">
-        <v>-16.09</v>
+        <v>31.51</v>
       </c>
       <c r="F21">
-        <v>748.66</v>
+        <v>718.94</v>
       </c>
       <c r="G21">
-        <v>-2.1</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2613,10 +2613,10 @@
         <v>100.0</v>
       </c>
       <c r="E23">
-        <v>228.53</v>
+        <v>232.18</v>
       </c>
       <c r="F23">
-        <v>228.53</v>
+        <v>232.18</v>
       </c>
       <c r="G23">
         <v>0.0</v>
@@ -2630,19 +2630,19 @@
         <v>6</v>
       </c>
       <c r="C24">
-        <v>782.91</v>
+        <v>772.09</v>
       </c>
       <c r="D24">
         <v>100.0</v>
       </c>
       <c r="E24">
-        <v>-11.44</v>
+        <v>-4.27</v>
       </c>
       <c r="F24">
-        <v>771.47</v>
+        <v>767.82</v>
       </c>
       <c r="G24">
-        <v>-1.5</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2676,13 +2676,13 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>279.51</v>
+        <v>236.24</v>
       </c>
       <c r="D26">
         <v>100.0</v>
       </c>
       <c r="E26">
-        <v>-279.51</v>
+        <v>-236.24</v>
       </c>
       <c r="F26">
         <v>0.0</v>
@@ -2699,19 +2699,19 @@
         <v>6</v>
       </c>
       <c r="C27">
-        <v>820.49</v>
+        <v>863.76</v>
       </c>
       <c r="D27">
         <v>100.0</v>
       </c>
       <c r="E27">
-        <v>47.1</v>
+        <v>-16.78</v>
       </c>
       <c r="F27">
-        <v>867.58</v>
+        <v>846.98</v>
       </c>
       <c r="G27">
-        <v>5.7</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2751,10 +2751,10 @@
         <v>100.0</v>
       </c>
       <c r="E29">
-        <v>140.05</v>
+        <v>175.39</v>
       </c>
       <c r="F29">
-        <v>140.05</v>
+        <v>175.39</v>
       </c>
       <c r="G29">
         <v>0.0</v>
@@ -2768,19 +2768,19 @@
         <v>6</v>
       </c>
       <c r="C30">
-        <v>817.13</v>
+        <v>833.99</v>
       </c>
       <c r="D30">
         <v>100.0</v>
       </c>
       <c r="E30">
-        <v>42.82</v>
+        <v>-9.38</v>
       </c>
       <c r="F30">
-        <v>859.95</v>
+        <v>824.61</v>
       </c>
       <c r="G30">
-        <v>5.2</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2837,19 +2837,19 @@
         <v>6</v>
       </c>
       <c r="C33">
-        <v>678.99</v>
+        <v>750.93</v>
       </c>
       <c r="D33">
         <v>50.0</v>
       </c>
       <c r="E33">
-        <v>142.24</v>
+        <v>6.01</v>
       </c>
       <c r="F33">
-        <v>821.23</v>
+        <v>756.93</v>
       </c>
       <c r="G33">
-        <v>20.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -2906,19 +2906,19 @@
         <v>6</v>
       </c>
       <c r="C36">
-        <v>714.39</v>
+        <v>718.36</v>
       </c>
       <c r="D36">
         <v>50.0</v>
       </c>
       <c r="E36">
-        <v>-8.67</v>
+        <v>-26.24</v>
       </c>
       <c r="F36">
-        <v>705.72</v>
+        <v>692.12</v>
       </c>
       <c r="G36">
-        <v>-1.2</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2975,19 +2975,19 @@
         <v>6</v>
       </c>
       <c r="C39">
-        <v>577.83</v>
+        <v>598.44</v>
       </c>
       <c r="D39">
         <v>50.0</v>
       </c>
       <c r="E39">
-        <v>60.17</v>
+        <v>-4.35</v>
       </c>
       <c r="F39">
-        <v>638.01</v>
+        <v>594.1</v>
       </c>
       <c r="G39">
-        <v>10.4</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -3044,19 +3044,19 @@
         <v>6</v>
       </c>
       <c r="C42">
-        <v>495.66</v>
+        <v>505.42</v>
       </c>
       <c r="D42">
         <v>50.0</v>
       </c>
       <c r="E42">
-        <v>-16.03</v>
+        <v>-8.52</v>
       </c>
       <c r="F42">
-        <v>479.63</v>
+        <v>496.9</v>
       </c>
       <c r="G42">
-        <v>-3.2</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -3113,19 +3113,19 @@
         <v>6</v>
       </c>
       <c r="C45">
-        <v>144.23</v>
+        <v>173.23</v>
       </c>
       <c r="D45">
         <v>50.0</v>
       </c>
       <c r="E45">
-        <v>61.96</v>
+        <v>78.29</v>
       </c>
       <c r="F45">
-        <v>206.19</v>
+        <v>251.52</v>
       </c>
       <c r="G45">
-        <v>43.0</v>
+        <v>45.2</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -3182,19 +3182,19 @@
         <v>6</v>
       </c>
       <c r="C48">
-        <v>246.59</v>
+        <v>154.29</v>
       </c>
       <c r="D48">
         <v>50.0</v>
       </c>
       <c r="E48">
-        <v>-27.32</v>
+        <v>27.94</v>
       </c>
       <c r="F48">
-        <v>219.27</v>
+        <v>182.23</v>
       </c>
       <c r="G48">
-        <v>-11.1</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -3251,19 +3251,19 @@
         <v>6</v>
       </c>
       <c r="C51">
-        <v>175.01</v>
+        <v>224.86</v>
       </c>
       <c r="D51">
         <v>50.0</v>
       </c>
       <c r="E51">
-        <v>74.16</v>
+        <v>16.63</v>
       </c>
       <c r="F51">
-        <v>249.17</v>
+        <v>241.49</v>
       </c>
       <c r="G51">
-        <v>42.4</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -3320,19 +3320,19 @@
         <v>6</v>
       </c>
       <c r="C54">
-        <v>263.52</v>
+        <v>290.0</v>
       </c>
       <c r="D54">
         <v>50.0</v>
       </c>
       <c r="E54">
-        <v>-2.82</v>
+        <v>6.64</v>
       </c>
       <c r="F54">
-        <v>260.7</v>
+        <v>296.63</v>
       </c>
       <c r="G54">
-        <v>-1.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -3346,7 +3346,7 @@
         <v>1500.0</v>
       </c>
       <c r="D55">
-        <v>100.0</v>
+        <v>50.0</v>
       </c>
       <c r="E55">
         <v>-0.0</v>
@@ -3369,7 +3369,7 @@
         <v>0.0</v>
       </c>
       <c r="D56">
-        <v>100.0</v>
+        <v>50.0</v>
       </c>
       <c r="E56">
         <v>-0.0</v>
@@ -3389,19 +3389,19 @@
         <v>6</v>
       </c>
       <c r="C57">
-        <v>320.79</v>
+        <v>356.34</v>
       </c>
       <c r="D57">
-        <v>100.0</v>
+        <v>50.0</v>
       </c>
       <c r="E57">
-        <v>-60.15</v>
+        <v>34.81</v>
       </c>
       <c r="F57">
-        <v>260.64</v>
+        <v>391.15</v>
       </c>
       <c r="G57">
-        <v>-18.8</v>
+        <v>9.8</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -3458,19 +3458,19 @@
         <v>6</v>
       </c>
       <c r="C60">
-        <v>440.43</v>
+        <v>419.43</v>
       </c>
       <c r="D60">
         <v>100.0</v>
       </c>
       <c r="E60">
-        <v>-41.63</v>
+        <v>-62.95</v>
       </c>
       <c r="F60">
-        <v>398.81</v>
+        <v>356.48</v>
       </c>
       <c r="G60">
-        <v>-9.5</v>
+        <v>-15.0</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -3510,10 +3510,10 @@
         <v>100.0</v>
       </c>
       <c r="E62">
-        <v>77.54</v>
+        <v>11.89</v>
       </c>
       <c r="F62">
-        <v>77.54</v>
+        <v>11.89</v>
       </c>
       <c r="G62">
         <v>0.0</v>
@@ -3527,19 +3527,19 @@
         <v>6</v>
       </c>
       <c r="C63">
-        <v>488.24</v>
+        <v>520.7</v>
       </c>
       <c r="D63">
         <v>100.0</v>
       </c>
       <c r="E63">
-        <v>-45.22</v>
+        <v>-9.07</v>
       </c>
       <c r="F63">
-        <v>443.02</v>
+        <v>511.63</v>
       </c>
       <c r="G63">
-        <v>-9.3</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -3573,19 +3573,19 @@
         <v>5</v>
       </c>
       <c r="C65">
-        <v>327.04</v>
+        <v>278.01</v>
       </c>
       <c r="D65">
         <v>100.0</v>
       </c>
       <c r="E65">
-        <v>-250.85</v>
+        <v>-264.54</v>
       </c>
       <c r="F65">
-        <v>76.19</v>
+        <v>13.47</v>
       </c>
       <c r="G65">
-        <v>-76.7</v>
+        <v>-95.2</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -3596,19 +3596,19 @@
         <v>6</v>
       </c>
       <c r="C66">
-        <v>594.54</v>
+        <v>589.19</v>
       </c>
       <c r="D66">
         <v>100.0</v>
       </c>
       <c r="E66">
-        <v>-70.73</v>
+        <v>-2.65</v>
       </c>
       <c r="F66">
-        <v>523.81</v>
+        <v>586.53</v>
       </c>
       <c r="G66">
-        <v>-11.9</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -3648,10 +3648,10 @@
         <v>100.0</v>
       </c>
       <c r="E68">
-        <v>293.2</v>
+        <v>309.01</v>
       </c>
       <c r="F68">
-        <v>293.2</v>
+        <v>309.01</v>
       </c>
       <c r="G68">
         <v>0.0</v>
@@ -3665,19 +3665,19 @@
         <v>6</v>
       </c>
       <c r="C69">
-        <v>370.18</v>
+        <v>392.11</v>
       </c>
       <c r="D69">
         <v>100.0</v>
       </c>
       <c r="E69">
-        <v>36.62</v>
+        <v>-1.12</v>
       </c>
       <c r="F69">
-        <v>406.8</v>
+        <v>390.99</v>
       </c>
       <c r="G69">
-        <v>9.9</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -3711,19 +3711,19 @@
         <v>5</v>
       </c>
       <c r="C71">
-        <v>377.53</v>
+        <v>305.16</v>
       </c>
       <c r="D71">
         <v>100.0</v>
       </c>
       <c r="E71">
-        <v>-74.23</v>
+        <v>63.5</v>
       </c>
       <c r="F71">
-        <v>303.3</v>
+        <v>368.66</v>
       </c>
       <c r="G71">
-        <v>-19.7</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -3734,19 +3734,19 @@
         <v>6</v>
       </c>
       <c r="C72">
-        <v>322.47</v>
+        <v>394.84</v>
       </c>
       <c r="D72">
         <v>100.0</v>
       </c>
       <c r="E72">
-        <v>74.23</v>
+        <v>-63.5</v>
       </c>
       <c r="F72">
-        <v>396.7</v>
+        <v>331.34</v>
       </c>
       <c r="G72">
-        <v>23.0</v>
+        <v>-16.1</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -3786,10 +3786,10 @@
         <v>100.0</v>
       </c>
       <c r="E74">
-        <v>434.22</v>
+        <v>513.08</v>
       </c>
       <c r="F74">
-        <v>434.22</v>
+        <v>513.08</v>
       </c>
       <c r="G74">
         <v>0.0</v>
@@ -3809,10 +3809,10 @@
         <v>100.0</v>
       </c>
       <c r="E75">
-        <v>365.78</v>
+        <v>286.92</v>
       </c>
       <c r="F75">
-        <v>365.78</v>
+        <v>286.92</v>
       </c>
       <c r="G75">
         <v>0.0</v>
@@ -3910,7 +3910,7 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>238.14</v>
+        <v>245.88</v>
       </c>
       <c r="D6">
         <v>50.0</v>
@@ -3919,7 +3919,7 @@
         <v>-0.0</v>
       </c>
       <c r="F6">
-        <v>238.14</v>
+        <v>245.88</v>
       </c>
       <c r="G6">
         <v>-0.0</v>
@@ -3979,19 +3979,19 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <v>123.64</v>
+        <v>217.5</v>
       </c>
       <c r="D9">
         <v>50.0</v>
       </c>
       <c r="E9">
-        <v>71.66</v>
+        <v>-8.14</v>
       </c>
       <c r="F9">
-        <v>195.3</v>
+        <v>209.36</v>
       </c>
       <c r="G9">
-        <v>58.0</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -4048,19 +4048,19 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>269.52</v>
+        <v>227.77</v>
       </c>
       <c r="D12">
         <v>50.0</v>
       </c>
       <c r="E12">
-        <v>96.08</v>
+        <v>42.92</v>
       </c>
       <c r="F12">
-        <v>365.6</v>
+        <v>270.69</v>
       </c>
       <c r="G12">
-        <v>35.6</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -4117,19 +4117,19 @@
         <v>6</v>
       </c>
       <c r="C15">
-        <v>195.1</v>
+        <v>283.9</v>
       </c>
       <c r="D15">
         <v>50.0</v>
       </c>
       <c r="E15">
-        <v>147.49</v>
+        <v>27.4</v>
       </c>
       <c r="F15">
-        <v>342.59</v>
+        <v>311.3</v>
       </c>
       <c r="G15">
-        <v>75.6</v>
+        <v>9.7</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -4186,19 +4186,19 @@
         <v>6</v>
       </c>
       <c r="C18">
-        <v>335.82</v>
+        <v>382.59</v>
       </c>
       <c r="D18">
         <v>50.0</v>
       </c>
       <c r="E18">
-        <v>-19.26</v>
+        <v>-36.27</v>
       </c>
       <c r="F18">
-        <v>316.56</v>
+        <v>346.32</v>
       </c>
       <c r="G18">
-        <v>-5.7</v>
+        <v>-9.5</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -4212,7 +4212,7 @@
         <v>1500.0</v>
       </c>
       <c r="D19">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E19">
         <v>-0.0</v>
@@ -4235,13 +4235,13 @@
         <v>0.0</v>
       </c>
       <c r="D20">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E20">
-        <v>-0.0</v>
+        <v>33.83</v>
       </c>
       <c r="F20">
-        <v>0.0</v>
+        <v>33.83</v>
       </c>
       <c r="G20">
         <v>0.0</v>
@@ -4255,19 +4255,19 @@
         <v>6</v>
       </c>
       <c r="C21">
-        <v>460.38</v>
+        <v>411.85</v>
       </c>
       <c r="D21">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E21">
-        <v>-35.74</v>
+        <v>-45.69</v>
       </c>
       <c r="F21">
-        <v>424.64</v>
+        <v>366.17</v>
       </c>
       <c r="G21">
-        <v>-7.8</v>
+        <v>-11.1</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -4307,10 +4307,10 @@
         <v>100.0</v>
       </c>
       <c r="E23">
-        <v>290.93</v>
+        <v>309.44</v>
       </c>
       <c r="F23">
-        <v>290.93</v>
+        <v>309.44</v>
       </c>
       <c r="G23">
         <v>0.0</v>
@@ -4324,19 +4324,19 @@
         <v>6</v>
       </c>
       <c r="C24">
-        <v>524.2</v>
+        <v>472.64</v>
       </c>
       <c r="D24">
         <v>100.0</v>
       </c>
       <c r="E24">
-        <v>-15.13</v>
+        <v>17.93</v>
       </c>
       <c r="F24">
-        <v>509.07</v>
+        <v>490.56</v>
       </c>
       <c r="G24">
-        <v>-2.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -4370,19 +4370,19 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>409.47</v>
+        <v>403.5</v>
       </c>
       <c r="D26">
         <v>100.0</v>
       </c>
       <c r="E26">
-        <v>-323.92</v>
+        <v>-397.37</v>
       </c>
       <c r="F26">
-        <v>85.54</v>
+        <v>6.13</v>
       </c>
       <c r="G26">
-        <v>-79.1</v>
+        <v>-98.5</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -4393,19 +4393,19 @@
         <v>6</v>
       </c>
       <c r="C27">
-        <v>590.53</v>
+        <v>596.5</v>
       </c>
       <c r="D27">
         <v>100.0</v>
       </c>
       <c r="E27">
-        <v>-76.08</v>
+        <v>-2.63</v>
       </c>
       <c r="F27">
-        <v>514.46</v>
+        <v>593.87</v>
       </c>
       <c r="G27">
-        <v>-12.9</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -4445,10 +4445,10 @@
         <v>100.0</v>
       </c>
       <c r="E29">
-        <v>307.19</v>
+        <v>293.78</v>
       </c>
       <c r="F29">
-        <v>307.19</v>
+        <v>293.78</v>
       </c>
       <c r="G29">
         <v>0.0</v>
@@ -4462,19 +4462,19 @@
         <v>6</v>
       </c>
       <c r="C30">
-        <v>340.31</v>
+        <v>415.84</v>
       </c>
       <c r="D30">
         <v>100.0</v>
       </c>
       <c r="E30">
-        <v>52.5</v>
+        <v>-9.62</v>
       </c>
       <c r="F30">
-        <v>392.81</v>
+        <v>406.22</v>
       </c>
       <c r="G30">
-        <v>15.4</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -4508,19 +4508,19 @@
         <v>5</v>
       </c>
       <c r="C32">
-        <v>222.29</v>
+        <v>237.09</v>
       </c>
       <c r="D32">
         <v>100.0</v>
       </c>
       <c r="E32">
-        <v>-215.89</v>
+        <v>-197.25</v>
       </c>
       <c r="F32">
-        <v>6.4</v>
+        <v>39.84</v>
       </c>
       <c r="G32">
-        <v>-97.1</v>
+        <v>-83.2</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -4531,19 +4531,19 @@
         <v>6</v>
       </c>
       <c r="C33">
-        <v>393.2</v>
+        <v>354.43</v>
       </c>
       <c r="D33">
         <v>100.0</v>
       </c>
       <c r="E33">
-        <v>-19.6</v>
+        <v>-14.27</v>
       </c>
       <c r="F33">
-        <v>373.6</v>
+        <v>340.16</v>
       </c>
       <c r="G33">
-        <v>-5.0</v>
+        <v>-4.0</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -4577,19 +4577,19 @@
         <v>5</v>
       </c>
       <c r="C35">
-        <v>464.8</v>
+        <v>498.92</v>
       </c>
       <c r="D35">
         <v>100.0</v>
       </c>
       <c r="E35">
-        <v>35.41</v>
+        <v>14.54</v>
       </c>
       <c r="F35">
-        <v>500.21</v>
+        <v>513.46</v>
       </c>
       <c r="G35">
-        <v>7.6</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -4600,19 +4600,19 @@
         <v>6</v>
       </c>
       <c r="C36">
-        <v>335.2</v>
+        <v>301.08</v>
       </c>
       <c r="D36">
         <v>100.0</v>
       </c>
       <c r="E36">
-        <v>-35.41</v>
+        <v>-14.54</v>
       </c>
       <c r="F36">
-        <v>299.79</v>
+        <v>286.54</v>
       </c>
       <c r="G36">
-        <v>-10.6</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -4646,19 +4646,19 @@
         <v>5</v>
       </c>
       <c r="C38">
-        <v>436.18</v>
+        <v>361.13</v>
       </c>
       <c r="D38">
         <v>100.0</v>
       </c>
       <c r="E38">
-        <v>-72.11</v>
+        <v>77.4</v>
       </c>
       <c r="F38">
-        <v>364.06</v>
+        <v>438.53</v>
       </c>
       <c r="G38">
-        <v>-16.5</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -4669,19 +4669,19 @@
         <v>6</v>
       </c>
       <c r="C39">
-        <v>263.82</v>
+        <v>338.87</v>
       </c>
       <c r="D39">
         <v>100.0</v>
       </c>
       <c r="E39">
-        <v>72.11</v>
+        <v>-77.4</v>
       </c>
       <c r="F39">
-        <v>335.94</v>
+        <v>261.47</v>
       </c>
       <c r="G39">
-        <v>27.3</v>
+        <v>-22.8</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -4715,19 +4715,19 @@
         <v>5</v>
       </c>
       <c r="C41">
-        <v>356.09</v>
+        <v>369.89</v>
       </c>
       <c r="D41">
         <v>100.0</v>
       </c>
       <c r="E41">
-        <v>-68.58</v>
+        <v>-39.13</v>
       </c>
       <c r="F41">
-        <v>287.5</v>
+        <v>330.76</v>
       </c>
       <c r="G41">
-        <v>-19.3</v>
+        <v>-10.6</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -4738,19 +4738,19 @@
         <v>6</v>
       </c>
       <c r="C42">
-        <v>243.91</v>
+        <v>230.11</v>
       </c>
       <c r="D42">
         <v>100.0</v>
       </c>
       <c r="E42">
-        <v>68.58</v>
+        <v>39.13</v>
       </c>
       <c r="F42">
-        <v>312.5</v>
+        <v>269.24</v>
       </c>
       <c r="G42">
-        <v>28.1</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -4784,19 +4784,19 @@
         <v>5</v>
       </c>
       <c r="C44">
-        <v>380.87</v>
+        <v>439.71</v>
       </c>
       <c r="D44">
         <v>100.0</v>
       </c>
       <c r="E44">
-        <v>-21.93</v>
+        <v>33.67</v>
       </c>
       <c r="F44">
-        <v>358.94</v>
+        <v>473.38</v>
       </c>
       <c r="G44">
-        <v>-5.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -4807,19 +4807,19 @@
         <v>6</v>
       </c>
       <c r="C45">
-        <v>319.13</v>
+        <v>260.29</v>
       </c>
       <c r="D45">
         <v>100.0</v>
       </c>
       <c r="E45">
-        <v>21.93</v>
+        <v>-33.67</v>
       </c>
       <c r="F45">
-        <v>341.06</v>
+        <v>226.62</v>
       </c>
       <c r="G45">
-        <v>6.9</v>
+        <v>-12.9</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -4853,19 +4853,19 @@
         <v>5</v>
       </c>
       <c r="C47">
-        <v>473.74</v>
+        <v>514.24</v>
       </c>
       <c r="D47">
         <v>100.0</v>
       </c>
       <c r="E47">
-        <v>58.33</v>
+        <v>-15.3</v>
       </c>
       <c r="F47">
-        <v>532.07</v>
+        <v>498.94</v>
       </c>
       <c r="G47">
-        <v>12.3</v>
+        <v>-3.0</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -4876,19 +4876,19 @@
         <v>6</v>
       </c>
       <c r="C48">
-        <v>226.26</v>
+        <v>185.76</v>
       </c>
       <c r="D48">
         <v>100.0</v>
       </c>
       <c r="E48">
-        <v>-58.33</v>
+        <v>15.3</v>
       </c>
       <c r="F48">
-        <v>167.93</v>
+        <v>201.06</v>
       </c>
       <c r="G48">
-        <v>-25.8</v>
+        <v>8.2</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -4922,19 +4922,19 @@
         <v>5</v>
       </c>
       <c r="C50">
-        <v>525.46</v>
+        <v>502.58</v>
       </c>
       <c r="D50">
         <v>100.0</v>
       </c>
       <c r="E50">
-        <v>-21.97</v>
+        <v>-10.48</v>
       </c>
       <c r="F50">
-        <v>503.48</v>
+        <v>492.1</v>
       </c>
       <c r="G50">
-        <v>-4.2</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -4945,19 +4945,19 @@
         <v>6</v>
       </c>
       <c r="C51">
-        <v>174.54</v>
+        <v>197.42</v>
       </c>
       <c r="D51">
         <v>100.0</v>
       </c>
       <c r="E51">
-        <v>21.97</v>
+        <v>10.48</v>
       </c>
       <c r="F51">
-        <v>196.52</v>
+        <v>207.9</v>
       </c>
       <c r="G51">
-        <v>12.6</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -4991,19 +4991,19 @@
         <v>5</v>
       </c>
       <c r="C53">
-        <v>192.39</v>
+        <v>225.53</v>
       </c>
       <c r="D53">
         <v>100.0</v>
       </c>
       <c r="E53">
-        <v>-64.01</v>
+        <v>-36.33</v>
       </c>
       <c r="F53">
-        <v>128.38</v>
+        <v>189.19</v>
       </c>
       <c r="G53">
-        <v>-33.3</v>
+        <v>-16.1</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -5014,19 +5014,19 @@
         <v>6</v>
       </c>
       <c r="C54">
-        <v>707.61</v>
+        <v>674.47</v>
       </c>
       <c r="D54">
         <v>100.0</v>
       </c>
       <c r="E54">
-        <v>64.01</v>
+        <v>36.33</v>
       </c>
       <c r="F54">
-        <v>771.62</v>
+        <v>710.81</v>
       </c>
       <c r="G54">
-        <v>9.0</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -5060,19 +5060,19 @@
         <v>5</v>
       </c>
       <c r="C56">
-        <v>160.05</v>
+        <v>212.32</v>
       </c>
       <c r="D56">
         <v>100.0</v>
       </c>
       <c r="E56">
-        <v>90.39</v>
+        <v>-28.05</v>
       </c>
       <c r="F56">
-        <v>250.44</v>
+        <v>184.26</v>
       </c>
       <c r="G56">
-        <v>56.5</v>
+        <v>-13.2</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -5083,19 +5083,19 @@
         <v>6</v>
       </c>
       <c r="C57">
-        <v>839.95</v>
+        <v>787.68</v>
       </c>
       <c r="D57">
         <v>100.0</v>
       </c>
       <c r="E57">
-        <v>-90.39</v>
+        <v>28.05</v>
       </c>
       <c r="F57">
-        <v>749.56</v>
+        <v>815.74</v>
       </c>
       <c r="G57">
-        <v>-10.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -5129,19 +5129,19 @@
         <v>5</v>
       </c>
       <c r="C59">
-        <v>276.34</v>
+        <v>228.74</v>
       </c>
       <c r="D59">
         <v>100.0</v>
       </c>
       <c r="E59">
-        <v>-3.05</v>
+        <v>66.56</v>
       </c>
       <c r="F59">
-        <v>273.3</v>
+        <v>295.3</v>
       </c>
       <c r="G59">
-        <v>-1.1</v>
+        <v>29.1</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -5152,19 +5152,19 @@
         <v>6</v>
       </c>
       <c r="C60">
-        <v>823.66</v>
+        <v>871.26</v>
       </c>
       <c r="D60">
         <v>100.0</v>
       </c>
       <c r="E60">
-        <v>3.05</v>
+        <v>-66.56</v>
       </c>
       <c r="F60">
-        <v>826.7</v>
+        <v>804.7</v>
       </c>
       <c r="G60">
-        <v>0.4</v>
+        <v>-7.6</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -5198,19 +5198,19 @@
         <v>5</v>
       </c>
       <c r="C62">
-        <v>216.98</v>
+        <v>218.91</v>
       </c>
       <c r="D62">
         <v>100.0</v>
       </c>
       <c r="E62">
-        <v>-11.06</v>
+        <v>6.72</v>
       </c>
       <c r="F62">
-        <v>205.92</v>
+        <v>225.62</v>
       </c>
       <c r="G62">
-        <v>-5.1</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -5221,19 +5221,19 @@
         <v>6</v>
       </c>
       <c r="C63">
-        <v>783.02</v>
+        <v>781.09</v>
       </c>
       <c r="D63">
         <v>100.0</v>
       </c>
       <c r="E63">
-        <v>11.06</v>
+        <v>-6.72</v>
       </c>
       <c r="F63">
-        <v>794.08</v>
+        <v>774.38</v>
       </c>
       <c r="G63">
-        <v>1.4</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -5290,19 +5290,19 @@
         <v>6</v>
       </c>
       <c r="C66">
-        <v>773.49</v>
+        <v>765.86</v>
       </c>
       <c r="D66">
         <v>50.0</v>
       </c>
       <c r="E66">
-        <v>8.96</v>
+        <v>-12.34</v>
       </c>
       <c r="F66">
-        <v>782.45</v>
+        <v>753.52</v>
       </c>
       <c r="G66">
-        <v>1.2</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -5359,19 +5359,19 @@
         <v>6</v>
       </c>
       <c r="C69">
-        <v>731.93</v>
+        <v>717.81</v>
       </c>
       <c r="D69">
         <v>50.0</v>
       </c>
       <c r="E69">
-        <v>-45.8</v>
+        <v>-48.82</v>
       </c>
       <c r="F69">
-        <v>686.13</v>
+        <v>669.0</v>
       </c>
       <c r="G69">
-        <v>-6.3</v>
+        <v>-6.8</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -5428,19 +5428,19 @@
         <v>6</v>
       </c>
       <c r="C72">
-        <v>518.81</v>
+        <v>624.31</v>
       </c>
       <c r="D72">
         <v>50.0</v>
       </c>
       <c r="E72">
-        <v>142.44</v>
+        <v>-25.69</v>
       </c>
       <c r="F72">
-        <v>661.25</v>
+        <v>598.62</v>
       </c>
       <c r="G72">
-        <v>27.5</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -5457,10 +5457,10 @@
         <v>30.0</v>
       </c>
       <c r="E73">
-        <v>1480.6</v>
+        <v>1470.66</v>
       </c>
       <c r="F73">
-        <v>1480.6</v>
+        <v>1470.66</v>
       </c>
       <c r="G73">
         <v>0.0</v>
@@ -5503,10 +5503,10 @@
         <v>30.0</v>
       </c>
       <c r="E75">
-        <v>519.4</v>
+        <v>529.34</v>
       </c>
       <c r="F75">
-        <v>519.4</v>
+        <v>529.34</v>
       </c>
       <c r="G75">
         <v>0.0</v>

</xml_diff>

<commit_message>
get latest rolling from laura working in jupyterlab, update filepath references to general form, use shared noise helper
</commit_message>
<xml_diff>
--- a/simple_market_clearing/clearing_analysis.xlsx
+++ b/simple_market_clearing/clearing_analysis.xlsx
@@ -479,7 +479,7 @@
         <v>0.0</v>
       </c>
       <c r="D4">
-        <v>61.73</v>
+        <v>100.0</v>
       </c>
       <c r="E4">
         <v>-0.0</v>
@@ -502,7 +502,7 @@
         <v>0.0</v>
       </c>
       <c r="D5">
-        <v>61.73</v>
+        <v>100.0</v>
       </c>
       <c r="E5">
         <v>-0.0</v>
@@ -525,7 +525,7 @@
         <v>0.0</v>
       </c>
       <c r="D6">
-        <v>61.73</v>
+        <v>100.0</v>
       </c>
       <c r="E6">
         <v>-0.0</v>
@@ -548,7 +548,7 @@
         <v>0.0</v>
       </c>
       <c r="D7">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E7">
         <v>1500.0</v>
@@ -571,7 +571,7 @@
         <v>0.0</v>
       </c>
       <c r="D8">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E8">
         <v>-0.0</v>
@@ -594,13 +594,13 @@
         <v>0.0</v>
       </c>
       <c r="D9">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E9">
-        <v>214.67</v>
+        <v>211.53</v>
       </c>
       <c r="F9">
-        <v>214.67</v>
+        <v>211.53</v>
       </c>
       <c r="G9">
         <v>0.0</v>
@@ -617,7 +617,7 @@
         <v>0.0</v>
       </c>
       <c r="D10">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E10">
         <v>1500.0</v>
@@ -640,7 +640,7 @@
         <v>0.0</v>
       </c>
       <c r="D11">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E11">
         <v>-0.0</v>
@@ -663,13 +663,13 @@
         <v>0.0</v>
       </c>
       <c r="D12">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E12">
-        <v>170.01</v>
+        <v>231.41</v>
       </c>
       <c r="F12">
-        <v>170.01</v>
+        <v>231.41</v>
       </c>
       <c r="G12">
         <v>0.0</v>
@@ -686,7 +686,7 @@
         <v>0.0</v>
       </c>
       <c r="D13">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E13">
         <v>1500.0</v>
@@ -709,7 +709,7 @@
         <v>0.0</v>
       </c>
       <c r="D14">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E14">
         <v>-0.0</v>
@@ -732,13 +732,13 @@
         <v>0.0</v>
       </c>
       <c r="D15">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E15">
-        <v>317.56</v>
+        <v>158.49</v>
       </c>
       <c r="F15">
-        <v>317.56</v>
+        <v>158.49</v>
       </c>
       <c r="G15">
         <v>0.0</v>
@@ -755,7 +755,7 @@
         <v>0.0</v>
       </c>
       <c r="D16">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E16">
         <v>1500.0</v>
@@ -778,7 +778,7 @@
         <v>0.0</v>
       </c>
       <c r="D17">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E17">
         <v>-0.0</v>
@@ -801,13 +801,13 @@
         <v>0.0</v>
       </c>
       <c r="D18">
-        <v>50.0</v>
+        <v>81.0</v>
       </c>
       <c r="E18">
-        <v>240.68</v>
+        <v>262.83</v>
       </c>
       <c r="F18">
-        <v>240.68</v>
+        <v>262.83</v>
       </c>
       <c r="G18">
         <v>0.0</v>
@@ -824,7 +824,7 @@
         <v>0.0</v>
       </c>
       <c r="D19">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E19">
         <v>1500.0</v>
@@ -847,13 +847,13 @@
         <v>0.0</v>
       </c>
       <c r="D20">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E20">
-        <v>-0.0</v>
+        <v>56.02</v>
       </c>
       <c r="F20">
-        <v>0.0</v>
+        <v>56.02</v>
       </c>
       <c r="G20">
         <v>0.0</v>
@@ -870,13 +870,13 @@
         <v>0.0</v>
       </c>
       <c r="D21">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E21">
-        <v>367.61</v>
+        <v>243.98</v>
       </c>
       <c r="F21">
-        <v>367.61</v>
+        <v>243.98</v>
       </c>
       <c r="G21">
         <v>0.0</v>
@@ -893,7 +893,7 @@
         <v>0.0</v>
       </c>
       <c r="D22">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E22">
         <v>1500.0</v>
@@ -916,7 +916,7 @@
         <v>0.0</v>
       </c>
       <c r="D23">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E23">
         <v>-0.0</v>
@@ -939,13 +939,13 @@
         <v>0.0</v>
       </c>
       <c r="D24">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E24">
-        <v>402.05</v>
+        <v>369.55</v>
       </c>
       <c r="F24">
-        <v>402.05</v>
+        <v>369.55</v>
       </c>
       <c r="G24">
         <v>0.0</v>
@@ -1011,10 +1011,10 @@
         <v>100.0</v>
       </c>
       <c r="E27">
-        <v>560.98</v>
+        <v>573.24</v>
       </c>
       <c r="F27">
-        <v>560.98</v>
+        <v>573.24</v>
       </c>
       <c r="G27">
         <v>0.0</v>
@@ -1057,10 +1057,10 @@
         <v>100.0</v>
       </c>
       <c r="E29">
-        <v>406.13</v>
+        <v>345.71</v>
       </c>
       <c r="F29">
-        <v>406.13</v>
+        <v>345.71</v>
       </c>
       <c r="G29">
         <v>0.0</v>
@@ -1080,10 +1080,10 @@
         <v>100.0</v>
       </c>
       <c r="E30">
-        <v>593.87</v>
+        <v>654.29</v>
       </c>
       <c r="F30">
-        <v>593.87</v>
+        <v>654.29</v>
       </c>
       <c r="G30">
         <v>0.0</v>
@@ -1126,10 +1126,10 @@
         <v>100.0</v>
       </c>
       <c r="E32">
-        <v>324.99</v>
+        <v>224.7</v>
       </c>
       <c r="F32">
-        <v>324.99</v>
+        <v>224.7</v>
       </c>
       <c r="G32">
         <v>0.0</v>
@@ -1149,10 +1149,10 @@
         <v>100.0</v>
       </c>
       <c r="E33">
-        <v>375.01</v>
+        <v>475.3</v>
       </c>
       <c r="F33">
-        <v>375.01</v>
+        <v>475.3</v>
       </c>
       <c r="G33">
         <v>0.0</v>
@@ -1195,10 +1195,10 @@
         <v>100.0</v>
       </c>
       <c r="E35">
-        <v>198.23</v>
+        <v>176.25</v>
       </c>
       <c r="F35">
-        <v>198.23</v>
+        <v>176.25</v>
       </c>
       <c r="G35">
         <v>0.0</v>
@@ -1218,10 +1218,10 @@
         <v>100.0</v>
       </c>
       <c r="E36">
-        <v>329.77</v>
+        <v>367.72</v>
       </c>
       <c r="F36">
-        <v>329.77</v>
+        <v>367.72</v>
       </c>
       <c r="G36">
         <v>0.0</v>
@@ -1264,10 +1264,10 @@
         <v>100.0</v>
       </c>
       <c r="E38">
-        <v>573.61</v>
+        <v>501.05</v>
       </c>
       <c r="F38">
-        <v>573.61</v>
+        <v>501.05</v>
       </c>
       <c r="G38">
         <v>0.0</v>
@@ -1287,10 +1287,10 @@
         <v>100.0</v>
       </c>
       <c r="E39">
-        <v>226.39</v>
+        <v>298.95</v>
       </c>
       <c r="F39">
-        <v>226.39</v>
+        <v>298.95</v>
       </c>
       <c r="G39">
         <v>0.0</v>
@@ -1333,10 +1333,10 @@
         <v>100.0</v>
       </c>
       <c r="E41">
-        <v>369.86</v>
+        <v>357.62</v>
       </c>
       <c r="F41">
-        <v>369.86</v>
+        <v>357.62</v>
       </c>
       <c r="G41">
         <v>0.0</v>
@@ -1356,10 +1356,10 @@
         <v>100.0</v>
       </c>
       <c r="E42">
-        <v>330.14</v>
+        <v>342.38</v>
       </c>
       <c r="F42">
-        <v>330.14</v>
+        <v>342.38</v>
       </c>
       <c r="G42">
         <v>0.0</v>
@@ -1402,10 +1402,10 @@
         <v>100.0</v>
       </c>
       <c r="E44">
-        <v>238.44</v>
+        <v>308.3</v>
       </c>
       <c r="F44">
-        <v>238.44</v>
+        <v>308.3</v>
       </c>
       <c r="G44">
         <v>0.0</v>
@@ -1425,10 +1425,10 @@
         <v>100.0</v>
       </c>
       <c r="E45">
-        <v>361.56</v>
+        <v>291.7</v>
       </c>
       <c r="F45">
-        <v>361.56</v>
+        <v>291.7</v>
       </c>
       <c r="G45">
         <v>0.0</v>
@@ -1471,10 +1471,10 @@
         <v>100.0</v>
       </c>
       <c r="E47">
-        <v>458.97</v>
+        <v>436.9</v>
       </c>
       <c r="F47">
-        <v>458.97</v>
+        <v>436.9</v>
       </c>
       <c r="G47">
         <v>0.0</v>
@@ -1494,10 +1494,10 @@
         <v>100.0</v>
       </c>
       <c r="E48">
-        <v>241.03</v>
+        <v>263.1</v>
       </c>
       <c r="F48">
-        <v>241.03</v>
+        <v>263.1</v>
       </c>
       <c r="G48">
         <v>0.0</v>
@@ -1540,10 +1540,10 @@
         <v>100.0</v>
       </c>
       <c r="E50">
-        <v>534.68</v>
+        <v>522.22</v>
       </c>
       <c r="F50">
-        <v>534.68</v>
+        <v>522.22</v>
       </c>
       <c r="G50">
         <v>0.0</v>
@@ -1563,10 +1563,10 @@
         <v>100.0</v>
       </c>
       <c r="E51">
-        <v>165.32</v>
+        <v>177.78</v>
       </c>
       <c r="F51">
-        <v>165.32</v>
+        <v>177.78</v>
       </c>
       <c r="G51">
         <v>0.0</v>
@@ -1609,10 +1609,10 @@
         <v>100.0</v>
       </c>
       <c r="E53">
-        <v>463.16</v>
+        <v>516.55</v>
       </c>
       <c r="F53">
-        <v>463.16</v>
+        <v>516.55</v>
       </c>
       <c r="G53">
         <v>0.0</v>
@@ -1632,10 +1632,10 @@
         <v>100.0</v>
       </c>
       <c r="E54">
-        <v>236.84</v>
+        <v>183.45</v>
       </c>
       <c r="F54">
-        <v>236.84</v>
+        <v>183.45</v>
       </c>
       <c r="G54">
         <v>0.0</v>
@@ -1678,10 +1678,10 @@
         <v>100.0</v>
       </c>
       <c r="E56">
-        <v>181.76</v>
+        <v>203.22</v>
       </c>
       <c r="F56">
-        <v>181.76</v>
+        <v>203.22</v>
       </c>
       <c r="G56">
         <v>0.0</v>
@@ -1701,10 +1701,10 @@
         <v>100.0</v>
       </c>
       <c r="E57">
-        <v>718.24</v>
+        <v>696.78</v>
       </c>
       <c r="F57">
-        <v>718.24</v>
+        <v>696.78</v>
       </c>
       <c r="G57">
         <v>0.0</v>
@@ -1770,10 +1770,10 @@
         <v>100.0</v>
       </c>
       <c r="E60">
-        <v>691.03</v>
+        <v>794.18</v>
       </c>
       <c r="F60">
-        <v>691.03</v>
+        <v>794.18</v>
       </c>
       <c r="G60">
         <v>0.0</v>
@@ -1816,10 +1816,10 @@
         <v>100.0</v>
       </c>
       <c r="E62">
-        <v>193.58</v>
+        <v>277.49</v>
       </c>
       <c r="F62">
-        <v>193.58</v>
+        <v>277.49</v>
       </c>
       <c r="G62">
         <v>0.0</v>
@@ -1839,10 +1839,10 @@
         <v>100.0</v>
       </c>
       <c r="E63">
-        <v>906.42</v>
+        <v>822.51</v>
       </c>
       <c r="F63">
-        <v>906.42</v>
+        <v>822.51</v>
       </c>
       <c r="G63">
         <v>0.0</v>
@@ -1885,10 +1885,10 @@
         <v>100.0</v>
       </c>
       <c r="E65">
-        <v>169.5</v>
+        <v>197.0</v>
       </c>
       <c r="F65">
-        <v>169.5</v>
+        <v>197.0</v>
       </c>
       <c r="G65">
         <v>0.0</v>
@@ -1908,10 +1908,10 @@
         <v>100.0</v>
       </c>
       <c r="E66">
-        <v>830.5</v>
+        <v>803.0</v>
       </c>
       <c r="F66">
-        <v>830.5</v>
+        <v>803.0</v>
       </c>
       <c r="G66">
         <v>0.0</v>
@@ -1977,10 +1977,10 @@
         <v>50.0</v>
       </c>
       <c r="E69">
-        <v>825.6</v>
+        <v>742.25</v>
       </c>
       <c r="F69">
-        <v>825.6</v>
+        <v>742.25</v>
       </c>
       <c r="G69">
         <v>0.0</v>
@@ -2046,10 +2046,10 @@
         <v>50.0</v>
       </c>
       <c r="E72">
-        <v>676.87</v>
+        <v>691.1</v>
       </c>
       <c r="F72">
-        <v>676.87</v>
+        <v>691.1</v>
       </c>
       <c r="G72">
         <v>0.0</v>
@@ -2115,10 +2115,10 @@
         <v>50.0</v>
       </c>
       <c r="E75">
-        <v>562.08</v>
+        <v>666.13</v>
       </c>
       <c r="F75">
-        <v>562.08</v>
+        <v>666.13</v>
       </c>
       <c r="G75">
         <v>0.0</v>
@@ -2193,7 +2193,7 @@
         <v>5</v>
       </c>
       <c r="C5">
-        <v>83.39</v>
+        <v>272.62</v>
       </c>
       <c r="D5">
         <v>100.0</v>
@@ -2202,7 +2202,7 @@
         <v>-0.0</v>
       </c>
       <c r="F5">
-        <v>83.39</v>
+        <v>272.62</v>
       </c>
       <c r="G5">
         <v>-0.0</v>
@@ -2216,7 +2216,7 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>339.47</v>
+        <v>226.04</v>
       </c>
       <c r="D6">
         <v>100.0</v>
@@ -2225,7 +2225,7 @@
         <v>-0.0</v>
       </c>
       <c r="F6">
-        <v>339.47</v>
+        <v>226.04</v>
       </c>
       <c r="G6">
         <v>-0.0</v>
@@ -2262,19 +2262,19 @@
         <v>5</v>
       </c>
       <c r="C8">
-        <v>421.71</v>
+        <v>318.92</v>
       </c>
       <c r="D8">
         <v>100.0</v>
       </c>
       <c r="E8">
-        <v>-239.91</v>
+        <v>-157.22</v>
       </c>
       <c r="F8">
-        <v>181.8</v>
+        <v>161.7</v>
       </c>
       <c r="G8">
-        <v>-56.9</v>
+        <v>-49.3</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2285,19 +2285,19 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <v>178.29</v>
+        <v>281.08</v>
       </c>
       <c r="D9">
         <v>100.0</v>
       </c>
       <c r="E9">
-        <v>51.36</v>
+        <v>-85.42</v>
       </c>
       <c r="F9">
-        <v>229.65</v>
+        <v>195.66</v>
       </c>
       <c r="G9">
-        <v>28.8</v>
+        <v>-30.4</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2331,19 +2331,19 @@
         <v>5</v>
       </c>
       <c r="C11">
-        <v>475.66</v>
+        <v>494.97</v>
       </c>
       <c r="D11">
         <v>100.0</v>
       </c>
       <c r="E11">
-        <v>-17.98</v>
+        <v>-64.08</v>
       </c>
       <c r="F11">
-        <v>457.68</v>
+        <v>430.9</v>
       </c>
       <c r="G11">
-        <v>-3.8</v>
+        <v>-12.9</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2354,19 +2354,19 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>224.34</v>
+        <v>205.03</v>
       </c>
       <c r="D12">
         <v>100.0</v>
       </c>
       <c r="E12">
-        <v>17.98</v>
+        <v>64.08</v>
       </c>
       <c r="F12">
-        <v>242.32</v>
+        <v>269.1</v>
       </c>
       <c r="G12">
-        <v>8.0</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2400,19 +2400,19 @@
         <v>5</v>
       </c>
       <c r="C14">
-        <v>557.42</v>
+        <v>462.11</v>
       </c>
       <c r="D14">
         <v>100.0</v>
       </c>
       <c r="E14">
-        <v>66.93</v>
+        <v>37.23</v>
       </c>
       <c r="F14">
-        <v>624.36</v>
+        <v>499.34</v>
       </c>
       <c r="G14">
-        <v>12.0</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2423,19 +2423,19 @@
         <v>6</v>
       </c>
       <c r="C15">
-        <v>142.58</v>
+        <v>237.89</v>
       </c>
       <c r="D15">
         <v>100.0</v>
       </c>
       <c r="E15">
-        <v>-66.93</v>
+        <v>-37.23</v>
       </c>
       <c r="F15">
-        <v>75.64</v>
+        <v>200.66</v>
       </c>
       <c r="G15">
-        <v>-46.9</v>
+        <v>-15.6</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2469,19 +2469,19 @@
         <v>5</v>
       </c>
       <c r="C17">
-        <v>454.01</v>
+        <v>497.35</v>
       </c>
       <c r="D17">
         <v>100.0</v>
       </c>
       <c r="E17">
-        <v>20.1</v>
+        <v>56.09</v>
       </c>
       <c r="F17">
-        <v>474.11</v>
+        <v>553.44</v>
       </c>
       <c r="G17">
-        <v>4.4</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2492,19 +2492,19 @@
         <v>6</v>
       </c>
       <c r="C18">
-        <v>245.99</v>
+        <v>202.65</v>
       </c>
       <c r="D18">
         <v>100.0</v>
       </c>
       <c r="E18">
-        <v>-20.1</v>
+        <v>-56.09</v>
       </c>
       <c r="F18">
-        <v>225.89</v>
+        <v>146.56</v>
       </c>
       <c r="G18">
-        <v>-8.2</v>
+        <v>-27.7</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -2538,19 +2538,19 @@
         <v>5</v>
       </c>
       <c r="C20">
-        <v>135.25</v>
+        <v>242.12</v>
       </c>
       <c r="D20">
         <v>100.0</v>
       </c>
       <c r="E20">
-        <v>16.09</v>
+        <v>-84.64</v>
       </c>
       <c r="F20">
-        <v>151.34</v>
+        <v>157.48</v>
       </c>
       <c r="G20">
-        <v>11.9</v>
+        <v>-35.0</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2561,19 +2561,19 @@
         <v>6</v>
       </c>
       <c r="C21">
-        <v>764.75</v>
+        <v>657.88</v>
       </c>
       <c r="D21">
         <v>100.0</v>
       </c>
       <c r="E21">
-        <v>-16.09</v>
+        <v>84.64</v>
       </c>
       <c r="F21">
-        <v>748.66</v>
+        <v>742.52</v>
       </c>
       <c r="G21">
-        <v>-2.1</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2613,10 +2613,10 @@
         <v>100.0</v>
       </c>
       <c r="E23">
-        <v>228.53</v>
+        <v>135.56</v>
       </c>
       <c r="F23">
-        <v>228.53</v>
+        <v>135.56</v>
       </c>
       <c r="G23">
         <v>0.0</v>
@@ -2630,19 +2630,19 @@
         <v>6</v>
       </c>
       <c r="C24">
-        <v>782.91</v>
+        <v>728.79</v>
       </c>
       <c r="D24">
         <v>100.0</v>
       </c>
       <c r="E24">
-        <v>-11.44</v>
+        <v>135.65</v>
       </c>
       <c r="F24">
-        <v>771.47</v>
+        <v>864.44</v>
       </c>
       <c r="G24">
-        <v>-1.5</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2676,13 +2676,13 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>279.51</v>
+        <v>226.27</v>
       </c>
       <c r="D26">
         <v>100.0</v>
       </c>
       <c r="E26">
-        <v>-279.51</v>
+        <v>-226.27</v>
       </c>
       <c r="F26">
         <v>0.0</v>
@@ -2699,19 +2699,19 @@
         <v>6</v>
       </c>
       <c r="C27">
-        <v>820.49</v>
+        <v>873.73</v>
       </c>
       <c r="D27">
         <v>100.0</v>
       </c>
       <c r="E27">
-        <v>47.1</v>
+        <v>34.4</v>
       </c>
       <c r="F27">
-        <v>867.58</v>
+        <v>908.14</v>
       </c>
       <c r="G27">
-        <v>5.7</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2751,10 +2751,10 @@
         <v>100.0</v>
       </c>
       <c r="E29">
-        <v>140.05</v>
+        <v>281.71</v>
       </c>
       <c r="F29">
-        <v>140.05</v>
+        <v>281.71</v>
       </c>
       <c r="G29">
         <v>0.0</v>
@@ -2768,19 +2768,19 @@
         <v>6</v>
       </c>
       <c r="C30">
-        <v>817.13</v>
+        <v>863.59</v>
       </c>
       <c r="D30">
         <v>100.0</v>
       </c>
       <c r="E30">
-        <v>42.82</v>
+        <v>-145.3</v>
       </c>
       <c r="F30">
-        <v>859.95</v>
+        <v>718.29</v>
       </c>
       <c r="G30">
-        <v>5.2</v>
+        <v>-16.8</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2837,19 +2837,19 @@
         <v>6</v>
       </c>
       <c r="C33">
-        <v>678.99</v>
+        <v>673.12</v>
       </c>
       <c r="D33">
         <v>50.0</v>
       </c>
       <c r="E33">
-        <v>142.24</v>
+        <v>153.28</v>
       </c>
       <c r="F33">
-        <v>821.23</v>
+        <v>826.4</v>
       </c>
       <c r="G33">
-        <v>20.9</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -2906,19 +2906,19 @@
         <v>6</v>
       </c>
       <c r="C36">
-        <v>714.39</v>
+        <v>683.01</v>
       </c>
       <c r="D36">
         <v>50.0</v>
       </c>
       <c r="E36">
-        <v>-8.67</v>
+        <v>9.25</v>
       </c>
       <c r="F36">
-        <v>705.72</v>
+        <v>692.26</v>
       </c>
       <c r="G36">
-        <v>-1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2975,19 +2975,19 @@
         <v>6</v>
       </c>
       <c r="C39">
-        <v>577.83</v>
+        <v>645.04</v>
       </c>
       <c r="D39">
         <v>50.0</v>
       </c>
       <c r="E39">
-        <v>60.17</v>
+        <v>31.73</v>
       </c>
       <c r="F39">
-        <v>638.01</v>
+        <v>676.77</v>
       </c>
       <c r="G39">
-        <v>10.4</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -3044,19 +3044,19 @@
         <v>6</v>
       </c>
       <c r="C42">
-        <v>495.66</v>
+        <v>513.31</v>
       </c>
       <c r="D42">
         <v>50.0</v>
       </c>
       <c r="E42">
-        <v>-16.03</v>
+        <v>-3.04</v>
       </c>
       <c r="F42">
-        <v>479.63</v>
+        <v>510.26</v>
       </c>
       <c r="G42">
-        <v>-3.2</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -3113,19 +3113,19 @@
         <v>6</v>
       </c>
       <c r="C45">
-        <v>144.23</v>
+        <v>124.85</v>
       </c>
       <c r="D45">
         <v>50.0</v>
       </c>
       <c r="E45">
-        <v>61.96</v>
+        <v>34.16</v>
       </c>
       <c r="F45">
-        <v>206.19</v>
+        <v>159.01</v>
       </c>
       <c r="G45">
-        <v>43.0</v>
+        <v>27.4</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -3182,19 +3182,19 @@
         <v>6</v>
       </c>
       <c r="C48">
-        <v>246.59</v>
+        <v>184.86</v>
       </c>
       <c r="D48">
         <v>50.0</v>
       </c>
       <c r="E48">
-        <v>-27.32</v>
+        <v>43.81</v>
       </c>
       <c r="F48">
-        <v>219.27</v>
+        <v>228.67</v>
       </c>
       <c r="G48">
-        <v>-11.1</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -3251,19 +3251,19 @@
         <v>6</v>
       </c>
       <c r="C51">
-        <v>175.01</v>
+        <v>290.64</v>
       </c>
       <c r="D51">
         <v>50.0</v>
       </c>
       <c r="E51">
-        <v>74.16</v>
+        <v>20.65</v>
       </c>
       <c r="F51">
-        <v>249.17</v>
+        <v>311.28</v>
       </c>
       <c r="G51">
-        <v>42.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -3320,19 +3320,19 @@
         <v>6</v>
       </c>
       <c r="C54">
-        <v>263.52</v>
+        <v>311.18</v>
       </c>
       <c r="D54">
         <v>50.0</v>
       </c>
       <c r="E54">
-        <v>-2.82</v>
+        <v>-18.51</v>
       </c>
       <c r="F54">
-        <v>260.7</v>
+        <v>292.67</v>
       </c>
       <c r="G54">
-        <v>-1.1</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -3389,19 +3389,19 @@
         <v>6</v>
       </c>
       <c r="C57">
-        <v>320.79</v>
+        <v>312.82</v>
       </c>
       <c r="D57">
         <v>100.0</v>
       </c>
       <c r="E57">
-        <v>-60.15</v>
+        <v>-40.33</v>
       </c>
       <c r="F57">
-        <v>260.64</v>
+        <v>272.49</v>
       </c>
       <c r="G57">
-        <v>-18.8</v>
+        <v>-12.9</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -3458,19 +3458,19 @@
         <v>6</v>
       </c>
       <c r="C60">
-        <v>440.43</v>
+        <v>304.72</v>
       </c>
       <c r="D60">
         <v>100.0</v>
       </c>
       <c r="E60">
-        <v>-41.63</v>
+        <v>60.36</v>
       </c>
       <c r="F60">
-        <v>398.81</v>
+        <v>365.08</v>
       </c>
       <c r="G60">
-        <v>-9.5</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -3510,10 +3510,10 @@
         <v>100.0</v>
       </c>
       <c r="E62">
-        <v>77.54</v>
+        <v>36.5</v>
       </c>
       <c r="F62">
-        <v>77.54</v>
+        <v>36.5</v>
       </c>
       <c r="G62">
         <v>0.0</v>
@@ -3527,19 +3527,19 @@
         <v>6</v>
       </c>
       <c r="C63">
-        <v>488.24</v>
+        <v>516.11</v>
       </c>
       <c r="D63">
         <v>100.0</v>
       </c>
       <c r="E63">
-        <v>-45.22</v>
+        <v>-10.17</v>
       </c>
       <c r="F63">
-        <v>443.02</v>
+        <v>505.94</v>
       </c>
       <c r="G63">
-        <v>-9.3</v>
+        <v>-2.0</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -3573,19 +3573,19 @@
         <v>5</v>
       </c>
       <c r="C65">
-        <v>327.04</v>
+        <v>354.94</v>
       </c>
       <c r="D65">
         <v>100.0</v>
       </c>
       <c r="E65">
-        <v>-250.85</v>
+        <v>-280.32</v>
       </c>
       <c r="F65">
-        <v>76.19</v>
+        <v>74.62</v>
       </c>
       <c r="G65">
-        <v>-76.7</v>
+        <v>-79.0</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -3596,19 +3596,19 @@
         <v>6</v>
       </c>
       <c r="C66">
-        <v>594.54</v>
+        <v>617.87</v>
       </c>
       <c r="D66">
         <v>100.0</v>
       </c>
       <c r="E66">
-        <v>-70.73</v>
+        <v>-92.49</v>
       </c>
       <c r="F66">
-        <v>523.81</v>
+        <v>525.38</v>
       </c>
       <c r="G66">
-        <v>-11.9</v>
+        <v>-15.0</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -3648,10 +3648,10 @@
         <v>100.0</v>
       </c>
       <c r="E68">
-        <v>293.2</v>
+        <v>230.28</v>
       </c>
       <c r="F68">
-        <v>293.2</v>
+        <v>230.28</v>
       </c>
       <c r="G68">
         <v>0.0</v>
@@ -3665,19 +3665,19 @@
         <v>6</v>
       </c>
       <c r="C69">
-        <v>370.18</v>
+        <v>386.36</v>
       </c>
       <c r="D69">
         <v>100.0</v>
       </c>
       <c r="E69">
-        <v>36.62</v>
+        <v>83.36</v>
       </c>
       <c r="F69">
-        <v>406.8</v>
+        <v>469.72</v>
       </c>
       <c r="G69">
-        <v>9.9</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -3711,19 +3711,19 @@
         <v>5</v>
       </c>
       <c r="C71">
-        <v>377.53</v>
+        <v>372.79</v>
       </c>
       <c r="D71">
         <v>100.0</v>
       </c>
       <c r="E71">
-        <v>-74.23</v>
+        <v>29.52</v>
       </c>
       <c r="F71">
-        <v>303.3</v>
+        <v>402.31</v>
       </c>
       <c r="G71">
-        <v>-19.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -3734,19 +3734,19 @@
         <v>6</v>
       </c>
       <c r="C72">
-        <v>322.47</v>
+        <v>327.21</v>
       </c>
       <c r="D72">
         <v>100.0</v>
       </c>
       <c r="E72">
-        <v>74.23</v>
+        <v>-29.52</v>
       </c>
       <c r="F72">
-        <v>396.7</v>
+        <v>297.69</v>
       </c>
       <c r="G72">
-        <v>23.0</v>
+        <v>-9.0</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -3786,10 +3786,10 @@
         <v>100.0</v>
       </c>
       <c r="E74">
-        <v>434.22</v>
+        <v>500.06</v>
       </c>
       <c r="F74">
-        <v>434.22</v>
+        <v>500.06</v>
       </c>
       <c r="G74">
         <v>0.0</v>
@@ -3809,10 +3809,10 @@
         <v>100.0</v>
       </c>
       <c r="E75">
-        <v>365.78</v>
+        <v>299.94</v>
       </c>
       <c r="F75">
-        <v>365.78</v>
+        <v>299.94</v>
       </c>
       <c r="G75">
         <v>0.0</v>
@@ -3910,7 +3910,7 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>238.14</v>
+        <v>127.23</v>
       </c>
       <c r="D6">
         <v>50.0</v>
@@ -3919,7 +3919,7 @@
         <v>-0.0</v>
       </c>
       <c r="F6">
-        <v>238.14</v>
+        <v>127.23</v>
       </c>
       <c r="G6">
         <v>-0.0</v>
@@ -3979,19 +3979,19 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <v>123.64</v>
+        <v>215.7</v>
       </c>
       <c r="D9">
         <v>50.0</v>
       </c>
       <c r="E9">
-        <v>71.66</v>
+        <v>73.25</v>
       </c>
       <c r="F9">
-        <v>195.3</v>
+        <v>288.95</v>
       </c>
       <c r="G9">
-        <v>58.0</v>
+        <v>34.0</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -4048,19 +4048,19 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>269.52</v>
+        <v>217.18</v>
       </c>
       <c r="D12">
         <v>50.0</v>
       </c>
       <c r="E12">
-        <v>96.08</v>
+        <v>45.72</v>
       </c>
       <c r="F12">
-        <v>365.6</v>
+        <v>262.9</v>
       </c>
       <c r="G12">
-        <v>35.6</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -4117,19 +4117,19 @@
         <v>6</v>
       </c>
       <c r="C15">
-        <v>195.1</v>
+        <v>359.08</v>
       </c>
       <c r="D15">
         <v>50.0</v>
       </c>
       <c r="E15">
-        <v>147.49</v>
+        <v>-176.57</v>
       </c>
       <c r="F15">
-        <v>342.59</v>
+        <v>182.52</v>
       </c>
       <c r="G15">
-        <v>75.6</v>
+        <v>-49.2</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -4186,19 +4186,19 @@
         <v>6</v>
       </c>
       <c r="C18">
-        <v>335.82</v>
+        <v>331.57</v>
       </c>
       <c r="D18">
         <v>50.0</v>
       </c>
       <c r="E18">
-        <v>-19.26</v>
+        <v>46.29</v>
       </c>
       <c r="F18">
-        <v>316.56</v>
+        <v>377.86</v>
       </c>
       <c r="G18">
-        <v>-5.7</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -4212,7 +4212,7 @@
         <v>1500.0</v>
       </c>
       <c r="D19">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E19">
         <v>-0.0</v>
@@ -4235,13 +4235,13 @@
         <v>0.0</v>
       </c>
       <c r="D20">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E20">
-        <v>-0.0</v>
+        <v>52.65</v>
       </c>
       <c r="F20">
-        <v>0.0</v>
+        <v>52.65</v>
       </c>
       <c r="G20">
         <v>0.0</v>
@@ -4255,19 +4255,19 @@
         <v>6</v>
       </c>
       <c r="C21">
-        <v>460.38</v>
+        <v>424.72</v>
       </c>
       <c r="D21">
-        <v>50.0</v>
+        <v>100.0</v>
       </c>
       <c r="E21">
-        <v>-35.74</v>
+        <v>-77.37</v>
       </c>
       <c r="F21">
-        <v>424.64</v>
+        <v>347.35</v>
       </c>
       <c r="G21">
-        <v>-7.8</v>
+        <v>-18.2</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -4307,10 +4307,10 @@
         <v>100.0</v>
       </c>
       <c r="E23">
-        <v>290.93</v>
+        <v>186.18</v>
       </c>
       <c r="F23">
-        <v>290.93</v>
+        <v>186.18</v>
       </c>
       <c r="G23">
         <v>0.0</v>
@@ -4324,19 +4324,19 @@
         <v>6</v>
       </c>
       <c r="C24">
-        <v>524.2</v>
+        <v>514.21</v>
       </c>
       <c r="D24">
         <v>100.0</v>
       </c>
       <c r="E24">
-        <v>-15.13</v>
+        <v>99.61</v>
       </c>
       <c r="F24">
-        <v>509.07</v>
+        <v>613.82</v>
       </c>
       <c r="G24">
-        <v>-2.9</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -4370,19 +4370,19 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>409.47</v>
+        <v>424.02</v>
       </c>
       <c r="D26">
         <v>100.0</v>
       </c>
       <c r="E26">
-        <v>-323.92</v>
+        <v>-376.61</v>
       </c>
       <c r="F26">
-        <v>85.54</v>
+        <v>47.42</v>
       </c>
       <c r="G26">
-        <v>-79.1</v>
+        <v>-88.8</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -4393,19 +4393,19 @@
         <v>6</v>
       </c>
       <c r="C27">
-        <v>590.53</v>
+        <v>575.98</v>
       </c>
       <c r="D27">
         <v>100.0</v>
       </c>
       <c r="E27">
-        <v>-76.08</v>
+        <v>-23.39</v>
       </c>
       <c r="F27">
-        <v>514.46</v>
+        <v>552.58</v>
       </c>
       <c r="G27">
-        <v>-12.9</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -4445,10 +4445,10 @@
         <v>100.0</v>
       </c>
       <c r="E29">
-        <v>307.19</v>
+        <v>291.4</v>
       </c>
       <c r="F29">
-        <v>307.19</v>
+        <v>291.4</v>
       </c>
       <c r="G29">
         <v>0.0</v>
@@ -4462,19 +4462,19 @@
         <v>6</v>
       </c>
       <c r="C30">
-        <v>340.31</v>
+        <v>353.3</v>
       </c>
       <c r="D30">
         <v>100.0</v>
       </c>
       <c r="E30">
-        <v>52.5</v>
+        <v>55.29</v>
       </c>
       <c r="F30">
-        <v>392.81</v>
+        <v>408.6</v>
       </c>
       <c r="G30">
-        <v>15.4</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -4508,19 +4508,19 @@
         <v>5</v>
       </c>
       <c r="C32">
-        <v>222.29</v>
+        <v>377.4</v>
       </c>
       <c r="D32">
         <v>100.0</v>
       </c>
       <c r="E32">
-        <v>-215.89</v>
+        <v>-315.38</v>
       </c>
       <c r="F32">
-        <v>6.4</v>
+        <v>62.02</v>
       </c>
       <c r="G32">
-        <v>-97.1</v>
+        <v>-83.6</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -4531,19 +4531,19 @@
         <v>6</v>
       </c>
       <c r="C33">
-        <v>393.2</v>
+        <v>235.1</v>
       </c>
       <c r="D33">
         <v>100.0</v>
       </c>
       <c r="E33">
-        <v>-19.6</v>
+        <v>82.89</v>
       </c>
       <c r="F33">
-        <v>373.6</v>
+        <v>317.98</v>
       </c>
       <c r="G33">
-        <v>-5.0</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -4577,19 +4577,19 @@
         <v>5</v>
       </c>
       <c r="C35">
-        <v>464.8</v>
+        <v>477.09</v>
       </c>
       <c r="D35">
         <v>100.0</v>
       </c>
       <c r="E35">
-        <v>35.41</v>
+        <v>24.16</v>
       </c>
       <c r="F35">
-        <v>500.21</v>
+        <v>501.25</v>
       </c>
       <c r="G35">
-        <v>7.6</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -4600,19 +4600,19 @@
         <v>6</v>
       </c>
       <c r="C36">
-        <v>335.2</v>
+        <v>322.91</v>
       </c>
       <c r="D36">
         <v>100.0</v>
       </c>
       <c r="E36">
-        <v>-35.41</v>
+        <v>-24.16</v>
       </c>
       <c r="F36">
-        <v>299.79</v>
+        <v>298.75</v>
       </c>
       <c r="G36">
-        <v>-10.6</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -4646,19 +4646,19 @@
         <v>5</v>
       </c>
       <c r="C38">
-        <v>436.18</v>
+        <v>435.18</v>
       </c>
       <c r="D38">
         <v>100.0</v>
       </c>
       <c r="E38">
-        <v>-72.11</v>
+        <v>-60.57</v>
       </c>
       <c r="F38">
-        <v>364.06</v>
+        <v>374.61</v>
       </c>
       <c r="G38">
-        <v>-16.5</v>
+        <v>-13.9</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -4669,19 +4669,19 @@
         <v>6</v>
       </c>
       <c r="C39">
-        <v>263.82</v>
+        <v>264.82</v>
       </c>
       <c r="D39">
         <v>100.0</v>
       </c>
       <c r="E39">
-        <v>72.11</v>
+        <v>60.57</v>
       </c>
       <c r="F39">
-        <v>335.94</v>
+        <v>325.39</v>
       </c>
       <c r="G39">
-        <v>27.3</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -4715,19 +4715,19 @@
         <v>5</v>
       </c>
       <c r="C41">
-        <v>356.09</v>
+        <v>325.47</v>
       </c>
       <c r="D41">
         <v>100.0</v>
       </c>
       <c r="E41">
-        <v>-68.58</v>
+        <v>52.88</v>
       </c>
       <c r="F41">
-        <v>287.5</v>
+        <v>378.35</v>
       </c>
       <c r="G41">
-        <v>-19.3</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -4738,19 +4738,19 @@
         <v>6</v>
       </c>
       <c r="C42">
-        <v>243.91</v>
+        <v>274.53</v>
       </c>
       <c r="D42">
         <v>100.0</v>
       </c>
       <c r="E42">
-        <v>68.58</v>
+        <v>-52.88</v>
       </c>
       <c r="F42">
-        <v>312.5</v>
+        <v>221.65</v>
       </c>
       <c r="G42">
-        <v>28.1</v>
+        <v>-19.3</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -4784,19 +4784,19 @@
         <v>5</v>
       </c>
       <c r="C44">
-        <v>380.87</v>
+        <v>428.26</v>
       </c>
       <c r="D44">
         <v>100.0</v>
       </c>
       <c r="E44">
-        <v>-21.93</v>
+        <v>23.23</v>
       </c>
       <c r="F44">
-        <v>358.94</v>
+        <v>451.48</v>
       </c>
       <c r="G44">
-        <v>-5.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -4807,19 +4807,19 @@
         <v>6</v>
       </c>
       <c r="C45">
-        <v>319.13</v>
+        <v>271.74</v>
       </c>
       <c r="D45">
         <v>100.0</v>
       </c>
       <c r="E45">
-        <v>21.93</v>
+        <v>-23.23</v>
       </c>
       <c r="F45">
-        <v>341.06</v>
+        <v>248.52</v>
       </c>
       <c r="G45">
-        <v>6.9</v>
+        <v>-8.5</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -4853,19 +4853,19 @@
         <v>5</v>
       </c>
       <c r="C47">
-        <v>473.74</v>
+        <v>527.72</v>
       </c>
       <c r="D47">
         <v>100.0</v>
       </c>
       <c r="E47">
-        <v>58.33</v>
+        <v>-21.92</v>
       </c>
       <c r="F47">
-        <v>532.07</v>
+        <v>505.8</v>
       </c>
       <c r="G47">
-        <v>12.3</v>
+        <v>-4.2</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -4876,19 +4876,19 @@
         <v>6</v>
       </c>
       <c r="C48">
-        <v>226.26</v>
+        <v>172.28</v>
       </c>
       <c r="D48">
         <v>100.0</v>
       </c>
       <c r="E48">
-        <v>-58.33</v>
+        <v>21.92</v>
       </c>
       <c r="F48">
-        <v>167.93</v>
+        <v>194.2</v>
       </c>
       <c r="G48">
-        <v>-25.8</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -4922,19 +4922,19 @@
         <v>5</v>
       </c>
       <c r="C50">
-        <v>525.46</v>
+        <v>501.45</v>
       </c>
       <c r="D50">
         <v>100.0</v>
       </c>
       <c r="E50">
-        <v>-21.97</v>
+        <v>-19.53</v>
       </c>
       <c r="F50">
-        <v>503.48</v>
+        <v>481.92</v>
       </c>
       <c r="G50">
-        <v>-4.2</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -4945,19 +4945,19 @@
         <v>6</v>
       </c>
       <c r="C51">
-        <v>174.54</v>
+        <v>198.55</v>
       </c>
       <c r="D51">
         <v>100.0</v>
       </c>
       <c r="E51">
-        <v>21.97</v>
+        <v>19.53</v>
       </c>
       <c r="F51">
-        <v>196.52</v>
+        <v>218.08</v>
       </c>
       <c r="G51">
-        <v>12.6</v>
+        <v>9.8</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -4991,19 +4991,19 @@
         <v>5</v>
       </c>
       <c r="C53">
-        <v>192.39</v>
+        <v>302.0</v>
       </c>
       <c r="D53">
         <v>100.0</v>
       </c>
       <c r="E53">
-        <v>-64.01</v>
+        <v>-85.29</v>
       </c>
       <c r="F53">
-        <v>128.38</v>
+        <v>216.72</v>
       </c>
       <c r="G53">
-        <v>-33.3</v>
+        <v>-28.2</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -5014,19 +5014,19 @@
         <v>6</v>
       </c>
       <c r="C54">
-        <v>707.61</v>
+        <v>598.0</v>
       </c>
       <c r="D54">
         <v>100.0</v>
       </c>
       <c r="E54">
-        <v>64.01</v>
+        <v>85.29</v>
       </c>
       <c r="F54">
-        <v>771.62</v>
+        <v>683.28</v>
       </c>
       <c r="G54">
-        <v>9.0</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -5060,19 +5060,19 @@
         <v>5</v>
       </c>
       <c r="C56">
-        <v>160.05</v>
+        <v>235.09</v>
       </c>
       <c r="D56">
         <v>100.0</v>
       </c>
       <c r="E56">
-        <v>90.39</v>
+        <v>-35.09</v>
       </c>
       <c r="F56">
-        <v>250.44</v>
+        <v>199.99</v>
       </c>
       <c r="G56">
-        <v>56.5</v>
+        <v>-14.9</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -5083,19 +5083,19 @@
         <v>6</v>
       </c>
       <c r="C57">
-        <v>839.95</v>
+        <v>764.91</v>
       </c>
       <c r="D57">
         <v>100.0</v>
       </c>
       <c r="E57">
-        <v>-90.39</v>
+        <v>35.09</v>
       </c>
       <c r="F57">
-        <v>749.56</v>
+        <v>800.01</v>
       </c>
       <c r="G57">
-        <v>-10.8</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -5129,19 +5129,19 @@
         <v>5</v>
       </c>
       <c r="C59">
-        <v>276.34</v>
+        <v>236.7</v>
       </c>
       <c r="D59">
         <v>100.0</v>
       </c>
       <c r="E59">
-        <v>-3.05</v>
+        <v>19.28</v>
       </c>
       <c r="F59">
-        <v>273.3</v>
+        <v>255.98</v>
       </c>
       <c r="G59">
-        <v>-1.1</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -5152,19 +5152,19 @@
         <v>6</v>
       </c>
       <c r="C60">
-        <v>823.66</v>
+        <v>863.3</v>
       </c>
       <c r="D60">
         <v>100.0</v>
       </c>
       <c r="E60">
-        <v>3.05</v>
+        <v>-19.28</v>
       </c>
       <c r="F60">
-        <v>826.7</v>
+        <v>844.02</v>
       </c>
       <c r="G60">
-        <v>0.4</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -5198,19 +5198,19 @@
         <v>5</v>
       </c>
       <c r="C62">
-        <v>216.98</v>
+        <v>92.45</v>
       </c>
       <c r="D62">
         <v>100.0</v>
       </c>
       <c r="E62">
-        <v>-11.06</v>
+        <v>53.71</v>
       </c>
       <c r="F62">
-        <v>205.92</v>
+        <v>146.16</v>
       </c>
       <c r="G62">
-        <v>-5.1</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -5221,19 +5221,19 @@
         <v>6</v>
       </c>
       <c r="C63">
-        <v>783.02</v>
+        <v>907.55</v>
       </c>
       <c r="D63">
         <v>100.0</v>
       </c>
       <c r="E63">
-        <v>11.06</v>
+        <v>-53.71</v>
       </c>
       <c r="F63">
-        <v>794.08</v>
+        <v>853.84</v>
       </c>
       <c r="G63">
-        <v>1.4</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -5290,19 +5290,19 @@
         <v>6</v>
       </c>
       <c r="C66">
-        <v>773.49</v>
+        <v>720.1</v>
       </c>
       <c r="D66">
         <v>50.0</v>
       </c>
       <c r="E66">
-        <v>8.96</v>
+        <v>83.26</v>
       </c>
       <c r="F66">
-        <v>782.45</v>
+        <v>803.35</v>
       </c>
       <c r="G66">
-        <v>1.2</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -5359,19 +5359,19 @@
         <v>6</v>
       </c>
       <c r="C69">
-        <v>731.93</v>
+        <v>659.63</v>
       </c>
       <c r="D69">
         <v>50.0</v>
       </c>
       <c r="E69">
-        <v>-45.8</v>
+        <v>51.09</v>
       </c>
       <c r="F69">
-        <v>686.13</v>
+        <v>710.72</v>
       </c>
       <c r="G69">
-        <v>-6.3</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -5428,19 +5428,19 @@
         <v>6</v>
       </c>
       <c r="C72">
-        <v>518.81</v>
+        <v>592.5</v>
       </c>
       <c r="D72">
         <v>50.0</v>
       </c>
       <c r="E72">
-        <v>142.44</v>
+        <v>-35.39</v>
       </c>
       <c r="F72">
-        <v>661.25</v>
+        <v>557.12</v>
       </c>
       <c r="G72">
-        <v>27.5</v>
+        <v>-6.0</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -5454,13 +5454,13 @@
         <v>0.0</v>
       </c>
       <c r="D73">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="E73">
-        <v>1480.6</v>
+        <v>1500.0</v>
       </c>
       <c r="F73">
-        <v>1480.6</v>
+        <v>1500.0</v>
       </c>
       <c r="G73">
         <v>0.0</v>
@@ -5477,7 +5477,7 @@
         <v>0.0</v>
       </c>
       <c r="D74">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="E74">
         <v>-0.0</v>
@@ -5500,13 +5500,13 @@
         <v>0.0</v>
       </c>
       <c r="D75">
-        <v>30.0</v>
+        <v>50.0</v>
       </c>
       <c r="E75">
-        <v>519.4</v>
+        <v>474.13</v>
       </c>
       <c r="F75">
-        <v>519.4</v>
+        <v>474.13</v>
       </c>
       <c r="G75">
         <v>0.0</v>

</xml_diff>